<commit_message>
Scenario rule fix (D2/D1/P), Snehal confirmed rater, Yen-Chu's answers
- Labeling kit: scenarios required for D2, D1 and P (matches taxonomy_v0
  codebook); workbook rebuilt; converter + irr Jaccard + RT20 updated
- Eval plan v1.2 note; README raters; Oct 18 minutes follow-up
- memory/11 + 09: Snehal rater, Yen-Chu transcripts by Oct 25, agent v1,
  model cost estimate

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/part3-metrics/labeling_round_1/labeling_workbook.xlsx
+++ b/docs/part3-metrics/labeling_round_1/labeling_workbook.xlsx
@@ -2501,10 +2501,10 @@
   </sheetData>
   <conditionalFormatting sqref="J3:J52">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND(LEN($J3)&gt;0,AND($I3&lt;&gt;"D1",$I3&lt;&gt;"D2"))</formula>
+      <formula>AND(LEN($J3)&gt;0,OR($I3="N",$I3="X"))</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="0">
-      <formula>AND(OR($I3="D1",$I3="D2"),LEN($J3)=0)</formula>
+      <formula>AND(OR($I3="D2",$I3="D1",$I3="P"),LEN($J3)=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -2514,7 +2514,7 @@
     <dataValidation sqref="I3:I52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Evidence level" prompt="D2 specific use · D1 general use · P plan · N no own use · X not substantive" type="list">
       <formula1>"D2,D1,P,N,X"</formula1>
     </dataValidation>
-    <dataValidation sqref="J3:J52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Scenarios" prompt="Only for D1/D2. Codes separated by ; e.g. CX;FRAUD" type="custom">
+    <dataValidation sqref="J3:J52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Scenarios" prompt="Required for D2/D1/P, blank for N/X. Codes separated by ; e.g. CX;FRAUD" type="custom">
       <formula1>TRUE</formula1>
     </dataValidation>
   </dataValidations>
@@ -2626,7 +2626,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>SCENARIOS (only for D1/D2; separate with ;)</t>
+          <t>SCENARIOS (required for D2, D1 and P; blank for N/X; separate with ;)</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Oct 23 checks: X rule for raters, keep agent results off main until Oct 27
- Cheat sheet, workbook, README: about_ai = N -> evidence X (X rule widened in #64)
- irr.py: a rater's about_ai = N counts as X, so labels made before the change still match
- README blind list now includes the agent output files (#66, #68)
- Eval plan: agent agreement so far is against the AI-assisted draft labels; 15 of the 50 sample passages are in the tuning set
- memory/09 entry and memory/11 updates

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/part3-metrics/labeling_round_1/labeling_workbook.xlsx
+++ b/docs/part3-metrics/labeling_round_1/labeling_workbook.xlsx
@@ -2599,7 +2599,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Not substantive: definition, acronym list, heading. e.g. 'AI: artificial intelligence.'</t>
+          <t>Not substantive: definition, acronym list, heading, or not actually about AI (about_ai = N). e.g. 'AI: artificial intelligence.'</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Mixed passage -&gt; highest level. 'may use / could include' -&gt; N. Other companies, criminals, the economy -&gt; N. Forward-looking-statement lists ('...technology changes, including AI') -&gt; N. Heading alone -&gt; X.</t>
+          <t>Mixed passage -&gt; highest level. 'may use / could include' -&gt; N. Other companies, criminals, the economy -&gt; N. Forward-looking-statement lists ('...technology changes, including AI') -&gt; N. Heading alone -&gt; X. about_ai = N -&gt; X.</t>
         </is>
       </c>
     </row>

</xml_diff>